<commit_message>
dodanie pliku z wykresami
</commit_message>
<xml_diff>
--- a/Wykresy.xlsx
+++ b/Wykresy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\studia_aisd\algorytmy_sortowania\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC88F6B5-67F6-4149-BF96-555224820697}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56B39A61-5BAE-493F-86A2-C5805A103D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{19E7D5CD-98A1-451F-9163-D7D48B512516}"/>
   </bookViews>
@@ -19,9 +19,6 @@
     <sheet name="MS" sheetId="4" r:id="rId4"/>
     <sheet name="QS" sheetId="5" r:id="rId5"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId6"/>
-  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -32,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="9">
   <si>
     <t>RANDOM</t>
   </si>
@@ -54,13 +51,19 @@
   <si>
     <t>V SHAPE</t>
   </si>
+  <si>
+    <t>LAST</t>
+  </si>
+  <si>
+    <t>MIDDLE</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="171" formatCode="0.00000"/>
+    <numFmt numFmtId="164" formatCode="0.00000"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -103,8 +106,8 @@
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="171" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
@@ -188,7 +191,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="pl-PL"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -3493,7 +3496,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>ASCENDING</c:v>
+                  <c:v>LAST</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -3589,7 +3592,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>DESCENDING</c:v>
+                  <c:v>MIDDLE</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -3673,198 +3676,6 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000002-368A-4447-9F1D-F10CFEFD7F11}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="3"/>
-          <c:order val="3"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>QS!$K$1</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>FLAT</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent4"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>QS!$L$3:$L$17</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="15"/>
-                <c:pt idx="0">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>3</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>4</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>5</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>6</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>8</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>9</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>10</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>11</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>12</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>13</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>14</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>15</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>QS!$K$3:$K$17</c:f>
-              <c:numCache>
-                <c:formatCode>0.00000</c:formatCode>
-                <c:ptCount val="15"/>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="1"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-368A-4447-9F1D-F10CFEFD7F11}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="4"/>
-          <c:order val="4"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>QS!$N$1</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>V SHAPE</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent5"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>QS!$O$3:$O$17</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="15"/>
-                <c:pt idx="0">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>3</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>4</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>5</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>6</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>8</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>9</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>10</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>11</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>12</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>13</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>14</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>15</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>QS!$N$3:$N$17</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="15"/>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="1"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-368A-4447-9F1D-F10CFEFD7F11}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7044,16 +6855,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>609599</xdr:colOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>552449</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
+      <xdr:rowOff>85725</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>304800</xdr:colOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>247650</xdr:colOff>
       <xdr:row>35</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -7081,148 +6892,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Arkusz1"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0">
-        <row r="1">
-          <cell r="B1" t="str">
-            <v>n</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="A3">
-            <v>1.2895630000002699E-2</v>
-          </cell>
-          <cell r="B3">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="A4">
-            <v>4.5536090000041399E-2</v>
-          </cell>
-          <cell r="B4">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5">
-            <v>0.10659839999998399</v>
-          </cell>
-          <cell r="B5">
-            <v>3</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6">
-            <v>0.17843498000002</v>
-          </cell>
-          <cell r="B6">
-            <v>4</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7">
-            <v>0.27907319000005298</v>
-          </cell>
-          <cell r="B7">
-            <v>5</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="A8">
-            <v>0.39907955999997202</v>
-          </cell>
-          <cell r="B8">
-            <v>6</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="A9">
-            <v>0.54504456000004198</v>
-          </cell>
-          <cell r="B9">
-            <v>7</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="A10">
-            <v>0.71580754000005897</v>
-          </cell>
-          <cell r="B10">
-            <v>8</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="A11">
-            <v>0.908800730000075</v>
-          </cell>
-          <cell r="B11">
-            <v>9</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="A12">
-            <v>1.1198589000000501</v>
-          </cell>
-          <cell r="B12">
-            <v>10</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="A13">
-            <v>1.35082415000006</v>
-          </cell>
-          <cell r="B13">
-            <v>11</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="A14">
-            <v>1.61096243000001</v>
-          </cell>
-          <cell r="B14">
-            <v>12</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="A15">
-            <v>1.89438412999998</v>
-          </cell>
-          <cell r="B15">
-            <v>13</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="A16">
-            <v>2.2099056500000098</v>
-          </cell>
-          <cell r="B16">
-            <v>14</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="A17">
-            <v>2.5968066699999302</v>
-          </cell>
-          <cell r="B17">
-            <v>15</v>
-          </cell>
-        </row>
-      </sheetData>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9399,23 +9068,19 @@
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
-      <c r="K1" s="1" t="s">
-        <v>5</v>
-      </c>
+      <c r="K1" s="1"/>
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
-      <c r="N1" s="1" t="s">
-        <v>6</v>
-      </c>
+      <c r="N1" s="1"/>
       <c r="O1" s="1"/>
     </row>
     <row r="2" spans="2:15" x14ac:dyDescent="0.25">
@@ -9438,18 +9103,10 @@
       <c r="I2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="K2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>2</v>
-      </c>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
     </row>
     <row r="3" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B3" s="3"/>
@@ -9466,13 +9123,9 @@
         <v>1</v>
       </c>
       <c r="K3" s="3"/>
-      <c r="L3" s="1">
-        <v>1</v>
-      </c>
+      <c r="L3" s="1"/>
       <c r="N3" s="3"/>
-      <c r="O3" s="1">
-        <v>1</v>
-      </c>
+      <c r="O3" s="1"/>
     </row>
     <row r="4" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B4" s="3"/>
@@ -9492,15 +9145,9 @@
         <v>2</v>
       </c>
       <c r="K4" s="3"/>
-      <c r="L4" s="1">
-        <f>L3+1</f>
-        <v>2</v>
-      </c>
+      <c r="L4" s="1"/>
       <c r="N4" s="3"/>
-      <c r="O4" s="1">
-        <f>O3+1</f>
-        <v>2</v>
-      </c>
+      <c r="O4" s="1"/>
     </row>
     <row r="5" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B5" s="3"/>
@@ -9519,15 +9166,9 @@
         <v>3</v>
       </c>
       <c r="K5" s="3"/>
-      <c r="L5" s="1">
-        <f t="shared" ref="L5:L17" si="2">L4+1</f>
-        <v>3</v>
-      </c>
+      <c r="L5" s="1"/>
       <c r="N5" s="3"/>
-      <c r="O5" s="1">
-        <f t="shared" ref="O5:O17" si="3">O4+1</f>
-        <v>3</v>
-      </c>
+      <c r="O5" s="1"/>
     </row>
     <row r="6" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B6" s="3"/>
@@ -9546,15 +9187,9 @@
         <v>4</v>
       </c>
       <c r="K6" s="3"/>
-      <c r="L6" s="1">
-        <f t="shared" si="2"/>
-        <v>4</v>
-      </c>
+      <c r="L6" s="1"/>
       <c r="N6" s="3"/>
-      <c r="O6" s="1">
-        <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
+      <c r="O6" s="1"/>
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B7" s="3"/>
@@ -9573,15 +9208,9 @@
         <v>5</v>
       </c>
       <c r="K7" s="3"/>
-      <c r="L7" s="1">
-        <f t="shared" si="2"/>
-        <v>5</v>
-      </c>
+      <c r="L7" s="1"/>
       <c r="N7" s="3"/>
-      <c r="O7" s="1">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
+      <c r="O7" s="1"/>
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B8" s="3"/>
@@ -9600,15 +9229,9 @@
         <v>6</v>
       </c>
       <c r="K8" s="3"/>
-      <c r="L8" s="1">
-        <f t="shared" si="2"/>
-        <v>6</v>
-      </c>
+      <c r="L8" s="1"/>
       <c r="N8" s="3"/>
-      <c r="O8" s="1">
-        <f t="shared" si="3"/>
-        <v>6</v>
-      </c>
+      <c r="O8" s="1"/>
     </row>
     <row r="9" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B9" s="3"/>
@@ -9627,15 +9250,9 @@
         <v>7</v>
       </c>
       <c r="K9" s="3"/>
-      <c r="L9" s="1">
-        <f t="shared" si="2"/>
-        <v>7</v>
-      </c>
+      <c r="L9" s="1"/>
       <c r="N9" s="3"/>
-      <c r="O9" s="1">
-        <f t="shared" si="3"/>
-        <v>7</v>
-      </c>
+      <c r="O9" s="1"/>
     </row>
     <row r="10" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B10" s="3"/>
@@ -9654,15 +9271,9 @@
         <v>8</v>
       </c>
       <c r="K10" s="3"/>
-      <c r="L10" s="1">
-        <f t="shared" si="2"/>
-        <v>8</v>
-      </c>
+      <c r="L10" s="1"/>
       <c r="N10" s="3"/>
-      <c r="O10" s="1">
-        <f t="shared" si="3"/>
-        <v>8</v>
-      </c>
+      <c r="O10" s="1"/>
     </row>
     <row r="11" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B11" s="3"/>
@@ -9681,15 +9292,9 @@
         <v>9</v>
       </c>
       <c r="K11" s="3"/>
-      <c r="L11" s="1">
-        <f t="shared" si="2"/>
-        <v>9</v>
-      </c>
+      <c r="L11" s="1"/>
       <c r="N11" s="3"/>
-      <c r="O11" s="1">
-        <f t="shared" si="3"/>
-        <v>9</v>
-      </c>
+      <c r="O11" s="1"/>
     </row>
     <row r="12" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B12" s="3"/>
@@ -9708,15 +9313,9 @@
         <v>10</v>
       </c>
       <c r="K12" s="3"/>
-      <c r="L12" s="1">
-        <f t="shared" si="2"/>
-        <v>10</v>
-      </c>
+      <c r="L12" s="1"/>
       <c r="N12" s="3"/>
-      <c r="O12" s="1">
-        <f t="shared" si="3"/>
-        <v>10</v>
-      </c>
+      <c r="O12" s="1"/>
     </row>
     <row r="13" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B13" s="3"/>
@@ -9735,15 +9334,9 @@
         <v>11</v>
       </c>
       <c r="K13" s="3"/>
-      <c r="L13" s="1">
-        <f t="shared" si="2"/>
-        <v>11</v>
-      </c>
+      <c r="L13" s="1"/>
       <c r="N13" s="3"/>
-      <c r="O13" s="1">
-        <f t="shared" si="3"/>
-        <v>11</v>
-      </c>
+      <c r="O13" s="1"/>
     </row>
     <row r="14" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B14" s="3"/>
@@ -9762,15 +9355,9 @@
         <v>12</v>
       </c>
       <c r="K14" s="3"/>
-      <c r="L14" s="1">
-        <f t="shared" si="2"/>
-        <v>12</v>
-      </c>
+      <c r="L14" s="1"/>
       <c r="N14" s="3"/>
-      <c r="O14" s="1">
-        <f t="shared" si="3"/>
-        <v>12</v>
-      </c>
+      <c r="O14" s="1"/>
     </row>
     <row r="15" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B15" s="3"/>
@@ -9789,15 +9376,9 @@
         <v>13</v>
       </c>
       <c r="K15" s="3"/>
-      <c r="L15" s="1">
-        <f t="shared" si="2"/>
-        <v>13</v>
-      </c>
+      <c r="L15" s="1"/>
       <c r="N15" s="3"/>
-      <c r="O15" s="1">
-        <f t="shared" si="3"/>
-        <v>13</v>
-      </c>
+      <c r="O15" s="1"/>
     </row>
     <row r="16" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B16" s="3"/>
@@ -9816,15 +9397,9 @@
         <v>14</v>
       </c>
       <c r="K16" s="3"/>
-      <c r="L16" s="1">
-        <f t="shared" si="2"/>
-        <v>14</v>
-      </c>
+      <c r="L16" s="1"/>
       <c r="N16" s="3"/>
-      <c r="O16" s="1">
-        <f t="shared" si="3"/>
-        <v>14</v>
-      </c>
+      <c r="O16" s="1"/>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B17" s="3"/>
@@ -9844,15 +9419,9 @@
         <v>15</v>
       </c>
       <c r="K17" s="3"/>
-      <c r="L17" s="1">
-        <f t="shared" si="2"/>
-        <v>15</v>
-      </c>
+      <c r="L17" s="1"/>
       <c r="N17" s="3"/>
-      <c r="O17" s="1">
-        <f t="shared" si="3"/>
-        <v>15</v>
-      </c>
+      <c r="O17" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
dodanie zawartości wykresów, część
</commit_message>
<xml_diff>
--- a/Wykresy.xlsx
+++ b/Wykresy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\studia_aisd\algorytmy_sortowania\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56B39A61-5BAE-493F-86A2-C5805A103D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29D2C96D-AF92-4490-96D4-7495EB7A3C1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{19E7D5CD-98A1-451F-9163-D7D48B512516}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{19E7D5CD-98A1-451F-9163-D7D48B512516}"/>
   </bookViews>
   <sheets>
     <sheet name="IS" sheetId="1" r:id="rId1"/>
@@ -281,49 +281,49 @@
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="0">
-                    <c:v>0,01290</c:v>
+                    <c:v>0,01203</c:v>
                   </c:pt>
                   <c:pt idx="1">
-                    <c:v>0,04554</c:v>
+                    <c:v>0,04735</c:v>
                   </c:pt>
                   <c:pt idx="2">
-                    <c:v>0,10660</c:v>
+                    <c:v>0,10191</c:v>
                   </c:pt>
                   <c:pt idx="3">
-                    <c:v>0,17843</c:v>
+                    <c:v>0,17270</c:v>
                   </c:pt>
                   <c:pt idx="4">
-                    <c:v>0,27907</c:v>
+                    <c:v>0,26500</c:v>
                   </c:pt>
                   <c:pt idx="5">
-                    <c:v>0,39908</c:v>
+                    <c:v>0,38173</c:v>
                   </c:pt>
                   <c:pt idx="6">
-                    <c:v>0,54504</c:v>
+                    <c:v>0,51715</c:v>
                   </c:pt>
                   <c:pt idx="7">
-                    <c:v>0,71581</c:v>
+                    <c:v>0,67669</c:v>
                   </c:pt>
                   <c:pt idx="8">
-                    <c:v>0,90880</c:v>
+                    <c:v>0,85694</c:v>
                   </c:pt>
                   <c:pt idx="9">
-                    <c:v>1,11986</c:v>
+                    <c:v>1,05383</c:v>
                   </c:pt>
                   <c:pt idx="10">
-                    <c:v>1,35082</c:v>
+                    <c:v>1,29811</c:v>
                   </c:pt>
                   <c:pt idx="11">
-                    <c:v>1,61096</c:v>
+                    <c:v>1,52764</c:v>
                   </c:pt>
                   <c:pt idx="12">
-                    <c:v>1,89438</c:v>
+                    <c:v>1,79703</c:v>
                   </c:pt>
                   <c:pt idx="13">
-                    <c:v>2,20991</c:v>
+                    <c:v>2,07821</c:v>
                   </c:pt>
                   <c:pt idx="14">
-                    <c:v>2,59681</c:v>
+                    <c:v>2,37830</c:v>
                   </c:pt>
                 </c:lvl>
               </c:multiLvlStrCache>
@@ -336,49 +336,49 @@
                 <c:formatCode>0.00000</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>1.2895630000002699E-2</c:v>
+                  <c:v>1.2026800000001E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.5536090000041399E-2</c:v>
+                  <c:v>4.7352119999999297E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.10659839999998399</c:v>
+                  <c:v>0.101906809999996</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.17843498000002</c:v>
+                  <c:v>0.172704049999998</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.27907319000005298</c:v>
+                  <c:v>0.265004980000003</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.39907955999997202</c:v>
+                  <c:v>0.38173197000000397</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.54504456000004198</c:v>
+                  <c:v>0.51714583999999997</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.71580754000005897</c:v>
+                  <c:v>0.67668937000000196</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.908800730000075</c:v>
+                  <c:v>0.85694406999999695</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1.1198589000000501</c:v>
+                  <c:v>1.0538272799999999</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.35082415000006</c:v>
+                  <c:v>1.29810537</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1.61096243000001</c:v>
+                  <c:v>1.5276361599999999</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1.89438412999998</c:v>
+                  <c:v>1.7970345999999999</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2.2099056500000098</c:v>
+                  <c:v>2.0782094199999999</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>2.5968066699999302</c:v>
+                  <c:v>2.3782967500000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -668,6 +668,51 @@
               <c:numCache>
                 <c:formatCode>0.00000</c:formatCode>
                 <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>1.0343999999804501E-4</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.65920000000596E-4</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.35649999996212E-4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3.1811000000061499E-4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5.1910999999904496E-4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4.8400999999671503E-4</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>5.6678000000260904E-4</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>6.2078999999926E-4</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>7.0693000000119298E-4</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>7.9233999999814796E-4</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>9.5499000000245297E-4</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>9.4290000000114501E-4</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.01204999999708E-3</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.09625999999707E-3</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1.17394000000103E-3</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -1096,57 +1141,106 @@
             <c:symbol val="none"/>
           </c:marker>
           <c:xVal>
-            <c:strRef>
+            <c:multiLvlStrRef>
               <c:f>SS!$B$3:$C$17</c:f>
-              <c:strCache>
+              <c:multiLvlStrCache>
                 <c:ptCount val="15"/>
-                <c:pt idx="0">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>3</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>4</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>5</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>6</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>8</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>9</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>10</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>11</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>12</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>13</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>14</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>15</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>1</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>2</c:v>
+                  </c:pt>
+                  <c:pt idx="2">
+                    <c:v>3</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>4</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
+                    <c:v>5</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>6</c:v>
+                  </c:pt>
+                  <c:pt idx="6">
+                    <c:v>7</c:v>
+                  </c:pt>
+                  <c:pt idx="7">
+                    <c:v>8</c:v>
+                  </c:pt>
+                  <c:pt idx="8">
+                    <c:v>9</c:v>
+                  </c:pt>
+                  <c:pt idx="9">
+                    <c:v>10</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
+                    <c:v>11</c:v>
+                  </c:pt>
+                  <c:pt idx="11">
+                    <c:v>12</c:v>
+                  </c:pt>
+                  <c:pt idx="12">
+                    <c:v>13</c:v>
+                  </c:pt>
+                  <c:pt idx="13">
+                    <c:v>14</c:v>
+                  </c:pt>
+                  <c:pt idx="14">
+                    <c:v>15</c:v>
+                  </c:pt>
+                </c:lvl>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>0,01138</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>0,04442</c:v>
+                  </c:pt>
+                  <c:pt idx="2">
+                    <c:v>0,09679</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>0,16176</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
+                    <c:v>0,25600</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>0,35798</c:v>
+                  </c:pt>
+                  <c:pt idx="6">
+                    <c:v>0,49104</c:v>
+                  </c:pt>
+                  <c:pt idx="7">
+                    <c:v>0,63820</c:v>
+                  </c:pt>
+                  <c:pt idx="8">
+                    <c:v>0,81029</c:v>
+                  </c:pt>
+                  <c:pt idx="9">
+                    <c:v>1,00392</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
+                    <c:v>1,21800</c:v>
+                  </c:pt>
+                  <c:pt idx="11">
+                    <c:v>1,45096</c:v>
+                  </c:pt>
+                  <c:pt idx="12">
+                    <c:v>1,70663</c:v>
+                  </c:pt>
+                  <c:pt idx="13">
+                    <c:v>1,99174</c:v>
+                  </c:pt>
+                  <c:pt idx="14">
+                    <c:v>2,43004</c:v>
+                  </c:pt>
+                </c:lvl>
+              </c:multiLvlStrCache>
+            </c:multiLvlStrRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
@@ -1154,6 +1248,51 @@
               <c:numCache>
                 <c:formatCode>0.00000</c:formatCode>
                 <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>1.13804100000038E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4.4423310000001902E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>9.6786580000002606E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.161760220000007</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.25599808999999102</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.35797905999999102</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.49104384999999401</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.638195540000003</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.81029029999999602</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.00392338</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.2179960299999899</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.45096204999999</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.70663114</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.99173796</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2.4300448299999902</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -1442,6 +1581,51 @@
               <c:numCache>
                 <c:formatCode>0.00000</c:formatCode>
                 <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>1.1810930000001401E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4.5579520000001102E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.102432369999996</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.17761743000000901</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.27528482000000098</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.39591920000000302</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.52693365999998598</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.69100402000001304</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.90792875999998102</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.1209079099999799</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.35179544999998</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.6097550999999799</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.88213537999999</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2.1775392799999902</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2.4898922799999998</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -1870,57 +2054,106 @@
             <c:symbol val="none"/>
           </c:marker>
           <c:xVal>
-            <c:strRef>
+            <c:multiLvlStrRef>
               <c:f>HS!$B$3:$C$17</c:f>
-              <c:strCache>
+              <c:multiLvlStrCache>
                 <c:ptCount val="15"/>
-                <c:pt idx="0">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>3</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>4</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>5</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>6</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>8</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>9</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>10</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>11</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>12</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>13</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>14</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>15</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>10</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>20</c:v>
+                  </c:pt>
+                  <c:pt idx="2">
+                    <c:v>30</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>40</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
+                    <c:v>50</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>60</c:v>
+                  </c:pt>
+                  <c:pt idx="6">
+                    <c:v>70</c:v>
+                  </c:pt>
+                  <c:pt idx="7">
+                    <c:v>80</c:v>
+                  </c:pt>
+                  <c:pt idx="8">
+                    <c:v>90</c:v>
+                  </c:pt>
+                  <c:pt idx="9">
+                    <c:v>100</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
+                    <c:v>110</c:v>
+                  </c:pt>
+                  <c:pt idx="11">
+                    <c:v>120</c:v>
+                  </c:pt>
+                  <c:pt idx="12">
+                    <c:v>130</c:v>
+                  </c:pt>
+                  <c:pt idx="13">
+                    <c:v>140</c:v>
+                  </c:pt>
+                  <c:pt idx="14">
+                    <c:v>150</c:v>
+                  </c:pt>
+                </c:lvl>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>0,02104</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>0,04179</c:v>
+                  </c:pt>
+                  <c:pt idx="2">
+                    <c:v>0,06579</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>0,08817</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
+                    <c:v>0,11055</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>0,13446</c:v>
+                  </c:pt>
+                  <c:pt idx="6">
+                    <c:v>0,16153</c:v>
+                  </c:pt>
+                  <c:pt idx="7">
+                    <c:v>0,18218</c:v>
+                  </c:pt>
+                  <c:pt idx="8">
+                    <c:v>0,20557</c:v>
+                  </c:pt>
+                  <c:pt idx="9">
+                    <c:v>0,23055</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
+                    <c:v>0,25660</c:v>
+                  </c:pt>
+                  <c:pt idx="11">
+                    <c:v>0,28242</c:v>
+                  </c:pt>
+                  <c:pt idx="12">
+                    <c:v>0,30764</c:v>
+                  </c:pt>
+                  <c:pt idx="13">
+                    <c:v>0,33841</c:v>
+                  </c:pt>
+                  <c:pt idx="14">
+                    <c:v>0,36236</c:v>
+                  </c:pt>
+                </c:lvl>
+              </c:multiLvlStrCache>
+            </c:multiLvlStrRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
@@ -1928,6 +2161,51 @@
               <c:numCache>
                 <c:formatCode>0.00000</c:formatCode>
                 <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>2.10359299999936E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4.1789509999989601E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6.5792329999999302E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8.81689399999913E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.110551459999987</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.13445716000001001</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.161532459999989</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.18217882999999799</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.205574060000003</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.23054614000000101</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.25660143000000002</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.28242096000001299</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.30764189999999803</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.33841027999999301</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.36235713000000902</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -2216,6 +2494,51 @@
               <c:numCache>
                 <c:formatCode>0.00000</c:formatCode>
                 <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>2.4259499999971E-3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4.34314999999969E-3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6.48232000000916E-3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8.7847700000111203E-3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.1156970000001799E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.3060779999977901E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.5788879999990901E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.8133170000009999E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2.0086530000003201E-2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2.2269469999991999E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2.4458189999995699E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2.6438289999987302E-2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2.8601709999998001E-2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>3.0908799999997402E-2</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>3.32464599999866E-2</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -2338,6 +2661,8 @@
         <c:scaling>
           <c:logBase val="2"/>
           <c:orientation val="minMax"/>
+          <c:max val="16"/>
+          <c:min val="1"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -7249,7 +7574,7 @@
     </row>
     <row r="3" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B3" s="2">
-        <v>1.2895630000002699E-2</v>
+        <v>1.2026800000001E-2</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -7262,7 +7587,9 @@
       <c r="I3" s="1">
         <v>1</v>
       </c>
-      <c r="K3" s="3"/>
+      <c r="K3" s="3">
+        <v>1.0343999999804501E-4</v>
+      </c>
       <c r="L3" s="1">
         <v>1</v>
       </c>
@@ -7273,7 +7600,7 @@
     </row>
     <row r="4" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B4" s="2">
-        <v>4.5536090000041399E-2</v>
+        <v>4.7352119999999297E-2</v>
       </c>
       <c r="C4">
         <f>C3+1</f>
@@ -7289,7 +7616,9 @@
         <f>I3+1</f>
         <v>2</v>
       </c>
-      <c r="K4" s="3"/>
+      <c r="K4" s="3">
+        <v>1.65920000000596E-4</v>
+      </c>
       <c r="L4" s="1">
         <f>L3+1</f>
         <v>2</v>
@@ -7302,7 +7631,7 @@
     </row>
     <row r="5" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B5" s="2">
-        <v>0.10659839999998399</v>
+        <v>0.101906809999996</v>
       </c>
       <c r="C5">
         <f t="shared" ref="C5:C17" si="0">C4+1</f>
@@ -7317,7 +7646,9 @@
         <f t="shared" ref="I5:I17" si="1">I4+1</f>
         <v>3</v>
       </c>
-      <c r="K5" s="3"/>
+      <c r="K5" s="3">
+        <v>2.35649999996212E-4</v>
+      </c>
       <c r="L5" s="1">
         <f t="shared" ref="L5:L17" si="2">L4+1</f>
         <v>3</v>
@@ -7330,7 +7661,7 @@
     </row>
     <row r="6" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B6" s="2">
-        <v>0.17843498000002</v>
+        <v>0.172704049999998</v>
       </c>
       <c r="C6">
         <f t="shared" si="0"/>
@@ -7345,7 +7676,9 @@
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="K6" s="3"/>
+      <c r="K6" s="3">
+        <v>3.1811000000061499E-4</v>
+      </c>
       <c r="L6" s="1">
         <f t="shared" si="2"/>
         <v>4</v>
@@ -7358,7 +7691,7 @@
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B7" s="2">
-        <v>0.27907319000005298</v>
+        <v>0.265004980000003</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
@@ -7373,7 +7706,9 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="K7" s="3"/>
+      <c r="K7" s="3">
+        <v>5.1910999999904496E-4</v>
+      </c>
       <c r="L7" s="1">
         <f t="shared" si="2"/>
         <v>5</v>
@@ -7386,7 +7721,7 @@
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B8" s="2">
-        <v>0.39907955999997202</v>
+        <v>0.38173197000000397</v>
       </c>
       <c r="C8">
         <f t="shared" si="0"/>
@@ -7401,7 +7736,9 @@
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="K8" s="3"/>
+      <c r="K8" s="3">
+        <v>4.8400999999671503E-4</v>
+      </c>
       <c r="L8" s="1">
         <f t="shared" si="2"/>
         <v>6</v>
@@ -7414,7 +7751,7 @@
     </row>
     <row r="9" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B9" s="2">
-        <v>0.54504456000004198</v>
+        <v>0.51714583999999997</v>
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
@@ -7429,7 +7766,9 @@
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="K9" s="3"/>
+      <c r="K9" s="3">
+        <v>5.6678000000260904E-4</v>
+      </c>
       <c r="L9" s="1">
         <f t="shared" si="2"/>
         <v>7</v>
@@ -7442,7 +7781,7 @@
     </row>
     <row r="10" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B10" s="2">
-        <v>0.71580754000005897</v>
+        <v>0.67668937000000196</v>
       </c>
       <c r="C10">
         <f t="shared" si="0"/>
@@ -7457,7 +7796,9 @@
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="K10" s="3"/>
+      <c r="K10" s="3">
+        <v>6.2078999999926E-4</v>
+      </c>
       <c r="L10" s="1">
         <f t="shared" si="2"/>
         <v>8</v>
@@ -7470,7 +7811,7 @@
     </row>
     <row r="11" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B11" s="2">
-        <v>0.908800730000075</v>
+        <v>0.85694406999999695</v>
       </c>
       <c r="C11">
         <f t="shared" si="0"/>
@@ -7485,7 +7826,9 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="K11" s="3"/>
+      <c r="K11" s="3">
+        <v>7.0693000000119298E-4</v>
+      </c>
       <c r="L11" s="1">
         <f t="shared" si="2"/>
         <v>9</v>
@@ -7498,7 +7841,7 @@
     </row>
     <row r="12" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B12" s="2">
-        <v>1.1198589000000501</v>
+        <v>1.0538272799999999</v>
       </c>
       <c r="C12">
         <f t="shared" si="0"/>
@@ -7513,7 +7856,9 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="K12" s="3"/>
+      <c r="K12" s="3">
+        <v>7.9233999999814796E-4</v>
+      </c>
       <c r="L12" s="1">
         <f t="shared" si="2"/>
         <v>10</v>
@@ -7526,7 +7871,7 @@
     </row>
     <row r="13" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B13" s="2">
-        <v>1.35082415000006</v>
+        <v>1.29810537</v>
       </c>
       <c r="C13">
         <f t="shared" si="0"/>
@@ -7541,7 +7886,9 @@
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
-      <c r="K13" s="3"/>
+      <c r="K13" s="3">
+        <v>9.5499000000245297E-4</v>
+      </c>
       <c r="L13" s="1">
         <f t="shared" si="2"/>
         <v>11</v>
@@ -7554,7 +7901,7 @@
     </row>
     <row r="14" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B14" s="2">
-        <v>1.61096243000001</v>
+        <v>1.5276361599999999</v>
       </c>
       <c r="C14">
         <f t="shared" si="0"/>
@@ -7569,7 +7916,9 @@
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="K14" s="3"/>
+      <c r="K14" s="3">
+        <v>9.4290000000114501E-4</v>
+      </c>
       <c r="L14" s="1">
         <f t="shared" si="2"/>
         <v>12</v>
@@ -7582,7 +7931,7 @@
     </row>
     <row r="15" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B15" s="2">
-        <v>1.89438412999998</v>
+        <v>1.7970345999999999</v>
       </c>
       <c r="C15">
         <f t="shared" si="0"/>
@@ -7597,7 +7946,9 @@
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
-      <c r="K15" s="3"/>
+      <c r="K15" s="3">
+        <v>1.01204999999708E-3</v>
+      </c>
       <c r="L15" s="1">
         <f t="shared" si="2"/>
         <v>13</v>
@@ -7610,7 +7961,7 @@
     </row>
     <row r="16" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B16" s="2">
-        <v>2.2099056500000098</v>
+        <v>2.0782094199999999</v>
       </c>
       <c r="C16">
         <f t="shared" si="0"/>
@@ -7625,7 +7976,9 @@
         <f t="shared" si="1"/>
         <v>14</v>
       </c>
-      <c r="K16" s="3"/>
+      <c r="K16" s="3">
+        <v>1.09625999999707E-3</v>
+      </c>
       <c r="L16" s="1">
         <f t="shared" si="2"/>
         <v>14</v>
@@ -7638,7 +7991,7 @@
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B17" s="2">
-        <v>2.5968066699999302</v>
+        <v>2.3782967500000001</v>
       </c>
       <c r="C17">
         <f t="shared" si="0"/>
@@ -7654,7 +8007,9 @@
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="K17" s="3"/>
+      <c r="K17" s="3">
+        <v>1.17394000000103E-3</v>
+      </c>
       <c r="L17" s="1">
         <f t="shared" si="2"/>
         <v>15</v>
@@ -7730,7 +8085,9 @@
       </c>
     </row>
     <row r="3" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B3" s="3"/>
+      <c r="B3" s="3">
+        <v>1.13804100000038E-2</v>
+      </c>
       <c r="C3">
         <v>1</v>
       </c>
@@ -7742,7 +8099,9 @@
       <c r="I3" s="1">
         <v>1</v>
       </c>
-      <c r="K3" s="3"/>
+      <c r="K3" s="3">
+        <v>1.1810930000001401E-2</v>
+      </c>
       <c r="L3" s="1">
         <v>1</v>
       </c>
@@ -7752,7 +8111,9 @@
       </c>
     </row>
     <row r="4" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B4" s="3"/>
+      <c r="B4" s="3">
+        <v>4.4423310000001902E-2</v>
+      </c>
       <c r="C4">
         <f>C3+1</f>
         <v>2</v>
@@ -7767,7 +8128,9 @@
         <f>I3+1</f>
         <v>2</v>
       </c>
-      <c r="K4" s="3"/>
+      <c r="K4" s="3">
+        <v>4.5579520000001102E-2</v>
+      </c>
       <c r="L4" s="1">
         <f>L3+1</f>
         <v>2</v>
@@ -7779,7 +8142,9 @@
       </c>
     </row>
     <row r="5" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B5" s="3"/>
+      <c r="B5" s="3">
+        <v>9.6786580000002606E-2</v>
+      </c>
       <c r="C5">
         <f t="shared" ref="C5:C17" si="0">C4+1</f>
         <v>3</v>
@@ -7793,7 +8158,9 @@
         <f t="shared" ref="I5:I17" si="1">I4+1</f>
         <v>3</v>
       </c>
-      <c r="K5" s="3"/>
+      <c r="K5" s="3">
+        <v>0.102432369999996</v>
+      </c>
       <c r="L5" s="1">
         <f t="shared" ref="L5:L17" si="2">L4+1</f>
         <v>3</v>
@@ -7805,7 +8172,9 @@
       </c>
     </row>
     <row r="6" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B6" s="3"/>
+      <c r="B6" s="3">
+        <v>0.161760220000007</v>
+      </c>
       <c r="C6">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -7819,7 +8188,9 @@
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="K6" s="3"/>
+      <c r="K6" s="3">
+        <v>0.17761743000000901</v>
+      </c>
       <c r="L6" s="1">
         <f t="shared" si="2"/>
         <v>4</v>
@@ -7831,7 +8202,9 @@
       </c>
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B7" s="3"/>
+      <c r="B7" s="3">
+        <v>0.25599808999999102</v>
+      </c>
       <c r="C7">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -7845,7 +8218,9 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="K7" s="3"/>
+      <c r="K7" s="3">
+        <v>0.27528482000000098</v>
+      </c>
       <c r="L7" s="1">
         <f t="shared" si="2"/>
         <v>5</v>
@@ -7857,7 +8232,9 @@
       </c>
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B8" s="3"/>
+      <c r="B8" s="3">
+        <v>0.35797905999999102</v>
+      </c>
       <c r="C8">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -7871,7 +8248,9 @@
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="K8" s="3"/>
+      <c r="K8" s="3">
+        <v>0.39591920000000302</v>
+      </c>
       <c r="L8" s="1">
         <f t="shared" si="2"/>
         <v>6</v>
@@ -7883,7 +8262,9 @@
       </c>
     </row>
     <row r="9" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B9" s="3"/>
+      <c r="B9" s="3">
+        <v>0.49104384999999401</v>
+      </c>
       <c r="C9">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -7897,7 +8278,9 @@
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="K9" s="3"/>
+      <c r="K9" s="3">
+        <v>0.52693365999998598</v>
+      </c>
       <c r="L9" s="1">
         <f t="shared" si="2"/>
         <v>7</v>
@@ -7909,7 +8292,9 @@
       </c>
     </row>
     <row r="10" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B10" s="3"/>
+      <c r="B10" s="3">
+        <v>0.638195540000003</v>
+      </c>
       <c r="C10">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -7923,7 +8308,9 @@
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="K10" s="3"/>
+      <c r="K10" s="3">
+        <v>0.69100402000001304</v>
+      </c>
       <c r="L10" s="1">
         <f t="shared" si="2"/>
         <v>8</v>
@@ -7935,7 +8322,9 @@
       </c>
     </row>
     <row r="11" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B11" s="3"/>
+      <c r="B11" s="3">
+        <v>0.81029029999999602</v>
+      </c>
       <c r="C11">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -7949,7 +8338,9 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="K11" s="3"/>
+      <c r="K11" s="3">
+        <v>0.90792875999998102</v>
+      </c>
       <c r="L11" s="1">
         <f t="shared" si="2"/>
         <v>9</v>
@@ -7961,7 +8352,9 @@
       </c>
     </row>
     <row r="12" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B12" s="3"/>
+      <c r="B12" s="3">
+        <v>1.00392338</v>
+      </c>
       <c r="C12">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -7975,7 +8368,9 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="K12" s="3"/>
+      <c r="K12" s="3">
+        <v>1.1209079099999799</v>
+      </c>
       <c r="L12" s="1">
         <f t="shared" si="2"/>
         <v>10</v>
@@ -7987,7 +8382,9 @@
       </c>
     </row>
     <row r="13" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B13" s="3"/>
+      <c r="B13" s="3">
+        <v>1.2179960299999899</v>
+      </c>
       <c r="C13">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -8001,7 +8398,9 @@
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
-      <c r="K13" s="3"/>
+      <c r="K13" s="3">
+        <v>1.35179544999998</v>
+      </c>
       <c r="L13" s="1">
         <f t="shared" si="2"/>
         <v>11</v>
@@ -8013,7 +8412,9 @@
       </c>
     </row>
     <row r="14" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B14" s="3"/>
+      <c r="B14" s="3">
+        <v>1.45096204999999</v>
+      </c>
       <c r="C14">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -8027,7 +8428,9 @@
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="K14" s="3"/>
+      <c r="K14" s="3">
+        <v>1.6097550999999799</v>
+      </c>
       <c r="L14" s="1">
         <f t="shared" si="2"/>
         <v>12</v>
@@ -8039,7 +8442,9 @@
       </c>
     </row>
     <row r="15" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B15" s="3"/>
+      <c r="B15" s="3">
+        <v>1.70663114</v>
+      </c>
       <c r="C15">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -8053,7 +8458,9 @@
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
-      <c r="K15" s="3"/>
+      <c r="K15" s="3">
+        <v>1.88213537999999</v>
+      </c>
       <c r="L15" s="1">
         <f t="shared" si="2"/>
         <v>13</v>
@@ -8065,7 +8472,9 @@
       </c>
     </row>
     <row r="16" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B16" s="3"/>
+      <c r="B16" s="3">
+        <v>1.99173796</v>
+      </c>
       <c r="C16">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -8079,7 +8488,9 @@
         <f t="shared" si="1"/>
         <v>14</v>
       </c>
-      <c r="K16" s="3"/>
+      <c r="K16" s="3">
+        <v>2.1775392799999902</v>
+      </c>
       <c r="L16" s="1">
         <f t="shared" si="2"/>
         <v>14</v>
@@ -8091,7 +8502,9 @@
       </c>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B17" s="3"/>
+      <c r="B17" s="3">
+        <v>2.4300448299999902</v>
+      </c>
       <c r="C17">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -8106,7 +8519,9 @@
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="K17" s="3"/>
+      <c r="K17" s="3">
+        <v>2.4898922799999998</v>
+      </c>
       <c r="L17" s="1">
         <f t="shared" si="2"/>
         <v>15</v>
@@ -8182,9 +8597,11 @@
       </c>
     </row>
     <row r="3" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B3" s="3"/>
+      <c r="B3" s="3">
+        <v>2.10359299999936E-2</v>
+      </c>
       <c r="C3">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E3" s="2"/>
       <c r="F3">
@@ -8194,7 +8611,9 @@
       <c r="I3" s="1">
         <v>1</v>
       </c>
-      <c r="K3" s="3"/>
+      <c r="K3" s="3">
+        <v>2.4259499999971E-3</v>
+      </c>
       <c r="L3" s="1">
         <v>1</v>
       </c>
@@ -8204,10 +8623,12 @@
       </c>
     </row>
     <row r="4" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B4" s="3"/>
+      <c r="B4" s="3">
+        <v>4.1789509999989601E-2</v>
+      </c>
       <c r="C4">
-        <f>C3+1</f>
-        <v>2</v>
+        <f>C3+10^1</f>
+        <v>20</v>
       </c>
       <c r="E4" s="2"/>
       <c r="F4">
@@ -8219,7 +8640,9 @@
         <f>I3+1</f>
         <v>2</v>
       </c>
-      <c r="K4" s="3"/>
+      <c r="K4" s="3">
+        <v>4.34314999999969E-3</v>
+      </c>
       <c r="L4" s="1">
         <f>L3+1</f>
         <v>2</v>
@@ -8231,10 +8654,12 @@
       </c>
     </row>
     <row r="5" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B5" s="3"/>
+      <c r="B5" s="3">
+        <v>6.5792329999999302E-2</v>
+      </c>
       <c r="C5">
-        <f t="shared" ref="C5:C17" si="0">C4+1</f>
-        <v>3</v>
+        <f t="shared" ref="C5:C17" si="0">C4+10^1</f>
+        <v>30</v>
       </c>
       <c r="E5" s="2"/>
       <c r="F5">
@@ -8245,7 +8670,9 @@
         <f t="shared" ref="I5:I17" si="1">I4+1</f>
         <v>3</v>
       </c>
-      <c r="K5" s="3"/>
+      <c r="K5" s="3">
+        <v>6.48232000000916E-3</v>
+      </c>
       <c r="L5" s="1">
         <f t="shared" ref="L5:L17" si="2">L4+1</f>
         <v>3</v>
@@ -8257,10 +8684,12 @@
       </c>
     </row>
     <row r="6" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B6" s="3"/>
+      <c r="B6" s="3">
+        <v>8.81689399999913E-2</v>
+      </c>
       <c r="C6">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="E6" s="2"/>
       <c r="F6">
@@ -8271,7 +8700,9 @@
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="K6" s="3"/>
+      <c r="K6" s="3">
+        <v>8.7847700000111203E-3</v>
+      </c>
       <c r="L6" s="1">
         <f t="shared" si="2"/>
         <v>4</v>
@@ -8283,10 +8714,12 @@
       </c>
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B7" s="3"/>
+      <c r="B7" s="3">
+        <v>0.110551459999987</v>
+      </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7">
@@ -8297,7 +8730,9 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="K7" s="3"/>
+      <c r="K7" s="3">
+        <v>1.1156970000001799E-2</v>
+      </c>
       <c r="L7" s="1">
         <f t="shared" si="2"/>
         <v>5</v>
@@ -8309,10 +8744,12 @@
       </c>
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B8" s="3"/>
+      <c r="B8" s="3">
+        <v>0.13445716000001001</v>
+      </c>
       <c r="C8">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>60</v>
       </c>
       <c r="E8" s="2"/>
       <c r="F8">
@@ -8323,7 +8760,9 @@
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="K8" s="3"/>
+      <c r="K8" s="3">
+        <v>1.3060779999977901E-2</v>
+      </c>
       <c r="L8" s="1">
         <f t="shared" si="2"/>
         <v>6</v>
@@ -8335,10 +8774,12 @@
       </c>
     </row>
     <row r="9" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B9" s="3"/>
+      <c r="B9" s="3">
+        <v>0.161532459999989</v>
+      </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>70</v>
       </c>
       <c r="E9" s="2"/>
       <c r="F9">
@@ -8349,7 +8790,9 @@
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="K9" s="3"/>
+      <c r="K9" s="3">
+        <v>1.5788879999990901E-2</v>
+      </c>
       <c r="L9" s="1">
         <f t="shared" si="2"/>
         <v>7</v>
@@ -8361,10 +8804,12 @@
       </c>
     </row>
     <row r="10" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B10" s="3"/>
+      <c r="B10" s="3">
+        <v>0.18217882999999799</v>
+      </c>
       <c r="C10">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>80</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10">
@@ -8375,7 +8820,9 @@
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="K10" s="3"/>
+      <c r="K10" s="3">
+        <v>1.8133170000009999E-2</v>
+      </c>
       <c r="L10" s="1">
         <f t="shared" si="2"/>
         <v>8</v>
@@ -8387,10 +8834,12 @@
       </c>
     </row>
     <row r="11" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B11" s="3"/>
+      <c r="B11" s="3">
+        <v>0.205574060000003</v>
+      </c>
       <c r="C11">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>90</v>
       </c>
       <c r="E11" s="2"/>
       <c r="F11">
@@ -8401,7 +8850,9 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="K11" s="3"/>
+      <c r="K11" s="3">
+        <v>2.0086530000003201E-2</v>
+      </c>
       <c r="L11" s="1">
         <f t="shared" si="2"/>
         <v>9</v>
@@ -8413,10 +8864,12 @@
       </c>
     </row>
     <row r="12" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B12" s="3"/>
+      <c r="B12" s="3">
+        <v>0.23054614000000101</v>
+      </c>
       <c r="C12">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="E12" s="2"/>
       <c r="F12">
@@ -8427,7 +8880,9 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="K12" s="3"/>
+      <c r="K12" s="3">
+        <v>2.2269469999991999E-2</v>
+      </c>
       <c r="L12" s="1">
         <f t="shared" si="2"/>
         <v>10</v>
@@ -8439,10 +8894,12 @@
       </c>
     </row>
     <row r="13" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B13" s="3"/>
+      <c r="B13" s="3">
+        <v>0.25660143000000002</v>
+      </c>
       <c r="C13">
         <f t="shared" si="0"/>
-        <v>11</v>
+        <v>110</v>
       </c>
       <c r="E13" s="2"/>
       <c r="F13">
@@ -8453,7 +8910,9 @@
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
-      <c r="K13" s="3"/>
+      <c r="K13" s="3">
+        <v>2.4458189999995699E-2</v>
+      </c>
       <c r="L13" s="1">
         <f t="shared" si="2"/>
         <v>11</v>
@@ -8465,10 +8924,12 @@
       </c>
     </row>
     <row r="14" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B14" s="3"/>
+      <c r="B14" s="3">
+        <v>0.28242096000001299</v>
+      </c>
       <c r="C14">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>120</v>
       </c>
       <c r="E14" s="2"/>
       <c r="F14">
@@ -8479,7 +8940,9 @@
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="K14" s="3"/>
+      <c r="K14" s="3">
+        <v>2.6438289999987302E-2</v>
+      </c>
       <c r="L14" s="1">
         <f t="shared" si="2"/>
         <v>12</v>
@@ -8491,10 +8954,12 @@
       </c>
     </row>
     <row r="15" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B15" s="3"/>
+      <c r="B15" s="3">
+        <v>0.30764189999999803</v>
+      </c>
       <c r="C15">
         <f t="shared" si="0"/>
-        <v>13</v>
+        <v>130</v>
       </c>
       <c r="E15" s="2"/>
       <c r="F15">
@@ -8505,7 +8970,9 @@
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
-      <c r="K15" s="3"/>
+      <c r="K15" s="3">
+        <v>2.8601709999998001E-2</v>
+      </c>
       <c r="L15" s="1">
         <f t="shared" si="2"/>
         <v>13</v>
@@ -8517,10 +8984,12 @@
       </c>
     </row>
     <row r="16" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B16" s="3"/>
+      <c r="B16" s="3">
+        <v>0.33841027999999301</v>
+      </c>
       <c r="C16">
         <f t="shared" si="0"/>
-        <v>14</v>
+        <v>140</v>
       </c>
       <c r="E16" s="2"/>
       <c r="F16">
@@ -8531,7 +9000,9 @@
         <f t="shared" si="1"/>
         <v>14</v>
       </c>
-      <c r="K16" s="3"/>
+      <c r="K16" s="3">
+        <v>3.0908799999997402E-2</v>
+      </c>
       <c r="L16" s="1">
         <f t="shared" si="2"/>
         <v>14</v>
@@ -8543,10 +9014,12 @@
       </c>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B17" s="3"/>
+      <c r="B17" s="3">
+        <v>0.36235713000000902</v>
+      </c>
       <c r="C17">
         <f t="shared" si="0"/>
-        <v>15</v>
+        <v>150</v>
       </c>
       <c r="E17" s="2"/>
       <c r="F17">
@@ -8558,7 +9031,9 @@
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="K17" s="3"/>
+      <c r="K17" s="3">
+        <v>3.32464599999866E-2</v>
+      </c>
       <c r="L17" s="1">
         <f t="shared" si="2"/>
         <v>15</v>

</xml_diff>